<commit_message>
Finish data-loss acceptance: atomic versions and export parity
Require expected_row_version on operator saves, bump versions on
milestones/import/jurisdiction changes, preserve drafts on conflict,
share list/export filters including q, reconcile sanitized fixtures,
and document Hostinger SQLite durability without touching hosted data.

Co-authored-by: tylerlfarr <tylerlfarr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/permit-tracker/server/fixtures/sanitized-source-workbook.xlsx
+++ b/permit-tracker/server/fixtures/sanitized-source-workbook.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,10 +426,10 @@
         <v>PW W/S Received</v>
       </c>
       <c r="G1" t="str">
-        <v/>
+        <v>Target Start Date</v>
       </c>
       <c r="H1" t="str">
-        <v/>
+        <v>Water &amp; Sewer Paid</v>
       </c>
       <c r="I1" t="str">
         <v/>
@@ -544,10 +544,10 @@
         <v>APPLY</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>10/17/26</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>4/5/26</v>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -597,16 +597,16 @@
         <v>4/3/26</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>4/4/26</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>4/6/26</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>11/21/26</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>4/7/26</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -662,7 +662,7 @@
         <v>LoCo Water Received</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>Target Start Date</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -780,7 +780,7 @@
         <v>na</v>
       </c>
       <c r="G7" t="str">
-        <v/>
+        <v>10/12/26</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -839,7 +839,7 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v/>
+        <v>12/6/26</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -878,9 +878,186 @@
         <v>ALTC-2026-00970</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Proj ID</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Lot</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Housetype</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Permit</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Utility Ordered</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Utility Received</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Target Start Date</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v>Permit time: Fairfax County sample</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>FFX1</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ID</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>Release</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Ordered</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Received</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Demo Fairfax Ridge</v>
+      </c>
+      <c r="B11" t="str">
+        <v>12</v>
+      </c>
+      <c r="C11" t="str">
+        <v>SF Detached</v>
+      </c>
+      <c r="D11" t="str">
+        <v>3/1/26</v>
+      </c>
+      <c r="E11" t="str">
+        <v>3/2/26</v>
+      </c>
+      <c r="F11" t="str">
+        <v>3/4/26</v>
+      </c>
+      <c r="G11" t="str">
+        <v>11/6/26</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v>BLDR-2026-00263</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implement Phase 2/3 workspace, authz, and coordinator fidelity
Add single-tenant workspace membership foundations, owner-gated
readiness rule writes, zero-row import rejection, no-lot/multi-permit
fixture coverage, incomplete masterfile/open-revision Attention surfaces,
and preview-actor binding — preserving Phase 1 DI/CAS/idempotency work.

Co-authored-by: tylerlfarr <tylerlfarr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/permit-tracker/server/fixtures/sanitized-source-workbook.xlsx
+++ b/permit-tracker/server/fixtures/sanitized-source-workbook.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -544,7 +544,7 @@
         <v>APPLY</v>
       </c>
       <c r="G3" t="str">
-        <v>10/17/26</v>
+        <v>10/18/26</v>
       </c>
       <c r="H3" t="str">
         <v>4/5/26</v>
@@ -603,7 +603,7 @@
         <v>4/6/26</v>
       </c>
       <c r="G4" t="str">
-        <v>11/21/26</v>
+        <v>11/22/26</v>
       </c>
       <c r="H4" t="str">
         <v>4/7/26</v>
@@ -780,7 +780,7 @@
         <v>na</v>
       </c>
       <c r="G7" t="str">
-        <v>10/12/26</v>
+        <v>10/13/26</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -839,7 +839,7 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>12/6/26</v>
+        <v>12/7/26</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -1016,7 +1016,7 @@
         <v>3/4/26</v>
       </c>
       <c r="G11" t="str">
-        <v>11/6/26</v>
+        <v>11/7/26</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -1055,9 +1055,245 @@
         <v>BLDR-2026-00263</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Demo Fairfax Ridge</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>Sales Office</v>
+      </c>
+      <c r="D12" t="str">
+        <v>3/5/26</v>
+      </c>
+      <c r="E12" t="str">
+        <v>3/6/26</v>
+      </c>
+      <c r="F12" t="str">
+        <v>3/7/26</v>
+      </c>
+      <c r="G12" t="str">
+        <v>11/17/26</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v>ALTC-2026-88001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Demo Fairfax Ridge</v>
+      </c>
+      <c r="B13" t="str">
+        <v>88</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Twin Pair</v>
+      </c>
+      <c r="D13" t="str">
+        <v>3/8/26</v>
+      </c>
+      <c r="E13" t="str">
+        <v>3/9/26</v>
+      </c>
+      <c r="F13" t="str">
+        <v>3/10/26</v>
+      </c>
+      <c r="G13" t="str">
+        <v>11/27/26</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v>ALTC-2026-88011 / ALTC-2026-88012</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Proj ID</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Lot</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Housetype</v>
+      </c>
+      <c r="D14" t="str">
+        <v>StartSheet</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Target</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Permit</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v>ID</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>